<commit_message>
Prompt and summary logic refined
</commit_message>
<xml_diff>
--- a/results/indicator_extract_10.xlsx
+++ b/results/indicator_extract_10.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B194"/>
+  <dimension ref="A1:B158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,1279 +436,1279 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Question</t>
+          <t>Indicator</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Producer-level activities are managed in a well-informed, effective and inclusive way.</t>
+          <t>Management has been adapted to include setting up committees, including for OHS.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.2.1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Effective and relevant data management supports improved decision-making.</t>
+          <t>Administration has been adapted with portions on CBA moved to 5.3.3 and clarification on applicability added.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.2.2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Continuous improvement is demonstrated in locally relevant sustainability areas.</t>
+          <t>Administration has been adapted to explicitly mention contracts as part of the mechanism for compliance.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.1.1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Capacities are strengthened through an inclusive and effective approach.</t>
+          <t>Management shows commitment to sustainable agriculture by allocating sufficient resources and staff to implement the Rainforest Alliance Sustainable Agriculture Standard. At least every three years, management evaluates its capacity for implementing the Rainforest Alliance Standard and demonstrates continuous improvement with subsequent assessments.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.2.1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>There is equal participation and recognition of women.</t>
+          <t>Management and producers comply with applicable laws relevant to the scope of the Rainforest Alliance Standard, including land use rights, environment, labor, human rights, FPIC, taxes, and anti-corruption issues.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.2.2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Locally relevant sustainability issues are addressed through collaborative action.</t>
+          <t>There is a comprehensive list of current service providers, suppliers, intermediaries, and subcontractors, with mechanisms in place to ensure compliance with the applicable requirements of the Standard for their activities within the scope of certification.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.2.3</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Measures are taken to improve climate change adaptation and mitigation.</t>
+          <t>An up-to-date registry of group members is maintained, with required information collected using the Group Member Registry form provided by the Rainforest Alliance.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.2.4</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Soil health is improved.</t>
+          <t>Up-to-date records of permanent and temporary workers are kept, containing full name, gender, year of birth, start and end dates of employment, wages including benefits, and additional information for workers with housing and young workers.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>1.2.5</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Quality and availability of water is optimised.</t>
+          <t>For permanent workers, up-to-date records are kept containing full name, gender, year of birth, and wages including benefits. For temporary workers, only the number of workers is required.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>1.2.6</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Biodiversity and natural habitats are conserved and enhanced.</t>
+          <t>Management ensures that when the Rainforest Alliance Standard requires to inform workers or group members, the information is provided in the predominant language(s) of the workers or group members.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>1.2.7</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Natural ecosystems and High Conservation Value areas are conserved.</t>
+          <t>An Agreement is in place between the group management and each group member signed by both parties, including obligations to comply with the Rainforest Alliance Standard, accept inspections and audits, guarantee certified product origin, right to appeal decisions, and agreement to share farm data.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>1.2.8</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>An Integrated Pest Management strategy is implemented.</t>
+          <t>Records for certification purposes and compliance are kept for a minimum of five years.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>1.2.9</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pesticides are registered and appropriately labelled.</t>
+          <t>An up-to-date map of the farm area is available, including farms, processing facilities, human habitation areas, schools, medical centers, natural ecosystems, riparian buffer zones, agroforestry systems, and protected areas, with risk areas identified and the date of the latest update displayed.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>1.2.10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Highly Hazardous Pesticides are actively phased out.</t>
+          <t>Geolocation data for all farm units with the certified crop is available for 100% of the farms, with at least 35% in the form of a GPS polygon, and all farm units having polygons by the second certification audit.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>1.2.11</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Environmental hazards of Highly Hazardous Pesticides are mitigated.</t>
+          <t>A polygon is available for each farm unit.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>1.3.1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Pesticides are handled and stored responsibly.</t>
+          <t>Management conducts a risk assessment in relation to the requirements in this Standard, by using the Risk Assessment Tool, at least every three years. The risk mitigation measures are included in the management plan.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>1.3.2</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Fibre quality is protected and enhanced.</t>
+          <t>Management develops a management plan that includes the goals and actions based on the Risk Assessment and self-assessment. For groups, the management plan is additionally based on the internal inspection. Management reports on the implementation of the management plan yearly. The management plan is updated yearly.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>1.3.3</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>An effective system identifies and addresses risks and incidents of labour rights violations.</t>
+          <t>Management provides group members and workers hired by the group with services based on the management plan. Services can include training, technical assistance, support in record keeping, access to inputs, awareness-raising activities, etc. Management documents the services provided.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>1.3.4</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Farmers and workers understand their labour rights.</t>
+          <t>Management provides workers with services based on the management plan. Services can include training, awareness-raising activities, etc. Management documents the services provided.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>There is no child labour, and the rights of children and young workers are protected.</t>
+          <t>Management has an internal inspection system in place to annually assess compliance of all actors within the scope of certification.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>5.4</t>
+          <t>1.4.1</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>There is no forced labour, and workers are freely employed.</t>
+          <t>Management has an internal inspection system in place to annually assess compliance of all actors within the scope of certification.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>1.4.2</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Farmers and workers have the right to freedom of association and collective bargaining.</t>
+          <t>Management conducts a yearly self-assessment to evaluate its own compliance, and that of all actors in its certification scope, with the relevant requirements in the Standard.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>1.4.3</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>There is no discrimination in labour practices.</t>
+          <t>An approval and sanction system is in place to ensure compliance of group members with the Rainforest Alliance Sustainable Agriculture Standard.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>5.7</t>
+          <t>1.5.1</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Workers are paid at least the minimum wage.</t>
+          <t>A Grievance Mechanism is in place that enables individuals, workers, communities, or civil society, including whistle-blowers, to raise complaints about the Certificate Holder’s activities.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>5.8</t>
+          <t>1.6.1</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Workers’ health and safety are protected.</t>
+          <t>Management commits to promoting gender equality by having a written statement communicated to group members or workers, appointing a committee responsible for the implementation, monitoring, and evaluation of measures that promote gender equality and women’s empowerment, and ensuring the committee includes at least one management representative with decision-making power and at least one person of each gender.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>5.9</t>
+          <t>1.6.2</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Workers have the right to a fair workplace, free of violence or harassment.</t>
+          <t>The responsible committee or person implements gender equality measures from the Risk Assessment and includes these measures in the management plan, raises awareness on gender equality and women’s empowerment with management and group staff at least annually, and is involved in remediation of cases on gender-based violence and gender-based discrimination per the Remediation Protocol.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>5.10</t>
+          <t>1.7.1</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Workers have clear work-related agreements and expectations.</t>
+          <t>Management collects accurate data on indicators relevant to the Rainforest Alliance Standard and reports this data through the Rainforest Alliance Certification Platform.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>2.1.1</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Measures are taken to improve sustainable livelihoods and resilience.</t>
+          <t>The total certified production and the certified production for each producer are estimated once a year based on a credible methodology for yield estimation of a representative sample of farms or farm units. The methodology and calculation are documented.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1.6.1</t>
+          <t>2.1.2</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>The Producer demonstrates collaboration or engagement with other relevant stakeholders on locally relevant sustainability issues.</t>
+          <t>Management takes stock annually of the total harvested certified production, the balance of products purchased, produced, sold, and in stock. In case the difference between estimated production and actual production is greater than 15%, a reasonable justification is given, and measures are taken to prevent such differences from occurring. For groups, the differences are checked and justified both on the group level and for the individual members.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1.1.1</t>
+          <t>2.1.3</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>A clear and locally relevant activity plan is developed and implemented for the Producer Unit, which is kept up to date, includes all activities, timelines, and responsibilities, and is reviewed at least annually considering monitoring findings.</t>
+          <t>Products certified against Rainforest Alliance Standard must be visually separated from non-certified products and from each other at all stages, including transport, storage, and processing.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1.1.2</t>
+          <t>2.1.4</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>A monitoring plan is developed and implemented that defines the data and methods used to identify risks of non-conformities, measure progress, and understand the effectiveness of Producer Unit activities. Data and information are recorded, and learnings shall be used to inform the activity plan in Indicator 1.1.1.</t>
+          <t>Management has mapped the product flow up to the final location of the certificate scope, including all intermediaries and activities carried out on the product.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1.1.3</t>
+          <t>2.1.5</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>A representative and inclusive sample of individuals involved in farm-level cotton production.</t>
+          <t>Certified products can be traced back to the certified farm(s) they were produced on.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1.1.3</t>
+          <t>2.1.5</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>A representative and inclusive sample of individuals involved in farm-level cotton production is consulted on their priorities and needs at least once a year. Key findings from this consultation are documented and considered in activity planning across all Principles and in setting priorities for continuous improvement.</t>
+          <t>Certified products can be traced back to the certified farm(s) they were produced on. Management keeps purchase and sales documents linked to physical deliveries from the certified, multi-certified and non-certified products, ensuring intermediaries do the same. The purchase and sales documents include date, product type, (percentage of) certified volume, group member details and, if relevant, traceability type. In case of group certification, group management ensures that group members receive a receipt for each delivery from the group member to the group or an intermediary, specifying name of group member, group member ID, date, product type and volume.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1.1.4</t>
+          <t>2.1.6</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>An effective management system is in place to plan and implement farming activities, enabling monitoring of progress against Better Cotton Indicators and continuous improvement targets, including the identification of non-conformities against standard requirements.</t>
+          <t>Shipments of certified products do not exceed the total production (for farms), purchase of certified products plus remaining stock balance from the previous year.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1.1.5</t>
+          <t>2.1.7</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>The Producer complies with all applicable laws and regulations.</t>
+          <t>There is no double selling of volumes. Once a volume is sold under a Rainforest Alliance Standard, conventional, another scheme or sustainability initiative, that volume is no longer available for sale.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1.1.6</t>
+          <t>2.1.8</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>The Producer takes measures to identify and mitigate any social and/or environmental risks that the farm operation poses to surrounding communities and land.</t>
+          <t>Group members keep sales receipts (electronic or physical), including name of group member, group member ID, date, product type, and volume.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1.2.1</t>
+          <t>2.1.9</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Accurate and complete Producer-level data is collected, validated, and reported in line with the Better Cotton Farm Data Requirements Document.</t>
+          <t>The correct methodology for the calculation of conversion factors is demonstrated and documented for each certified product and reflected accordingly in the traceability platform. Applicable for large farms in a group, if they have processing as part of the scope.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>2.1.10</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Accurate and complete farm-level data is collected, validated, and recorded in line with the Better Cotton Farm Data Requirements Document.</t>
+          <t>Equipment used to measure the weight or volume of the certified product is calibrated annually.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1.3.1</t>
+          <t>2.2.1</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Specific focus areas and respective three-year targets for continuous improvement are set, and annual activities to work towards those targets are fully included and implemented as part of the overall activity and monitoring planning and implementation.</t>
+          <t>Any activity related to the certified volume (such as redeeming, removing, selling, purchasing, confirming, etc.) must be recorded in the Rainforest Alliance traceability platform within two weeks after the end of the quarter in which the activity took place.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1.1.1</t>
+          <t>2.2.2</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Continuous improvement targets, activities, and monitoring are integrated into the PU’s overall planning and monitoring systems.</t>
+          <t>Buyers of Rainforest Alliance Certified products regularly verify that transactions in the traceability platform match invoices for certified products.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1.1.2</t>
+          <t>2.2.3</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Continuous improvement targets, activities, and monitoring are integrated into the PU’s overall planning and monitoring systems.</t>
+          <t>Approval is obtained prior to the on- and off-pack use of public-facing claims. There is evidence that any Rainforest Alliance claim made is valid and complies with Rainforest Alliance Certification Program Requirements.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1.3.2</t>
+          <t>2.2.4</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Specific and locally relevant sustainability targets are identified for continuous improvement, activities to achieve those targets are implemented, and progress is monitored as part of the overall management system.</t>
+          <t>Royalty is paid in full without any tax deductions, according to the payment terms set forth in the License Agreement, Terms and Conditions and/or the invoice.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>2.3.1</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>An effective programme is implemented to strengthen capacities of individuals involved in farm-level cotton production, focusing on locally relevant practices and innovations.</t>
+          <t>Volumes are only converted for processes that can occur in reality; product conversion cannot revert to a previous product.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>1.4.2</t>
+          <t>2.3.2</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Training and other related activities are designed to be inclusive and equally accessible to everyone who may benefit.</t>
+          <t>Volumes sold as mass balance are 100% covered by volumes purchased as certified. A negative volume balance is not permitted at any time.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>1.4.3</t>
+          <t>2.3.3</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Participants understand the relevance and benefits of knowledge, skills and practices promoted through training and other related activities.</t>
+          <t>Mass balance volumes must always be accompanied by a physical shipment when transferred between Certificate Holders. Volume trading without a physical shipment is only allowed between sites under the same certificate.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>1.1.2</t>
+          <t>2.3.4</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Producer Management should monitor changes in knowledge, attitudes, and practices directly and ensure that lessons learnt are used to inform adjustments in content, approaches, and tools for training and related activities.</t>
+          <t>Volumes sold as certified meet the minimum percentage requirements for origin information. This requirement is only applicable for cocoa mass balance products for which origin matching rules are required.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>1.4.4</t>
+          <t>2.3.5</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>An effective programme is implemented to strengthen capacities of workers. Training and related activities focus on locally relevant practices and innovations, are informed by consultation with workers and feedback loops from previous training, use effective approaches and tools, and are designed to be inclusive and equally accessible to all workers who may benefit.</t>
+          <t>Purchase and sales documentation for volumes sold as certified must include origin information to country level for both incoming certified and non-certified volumes. This is only applicable for cocoa mass balance products for which origin matching rules are required.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>1.5.1</t>
+          <t>3.1.1</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>An individual Gender Lead or Gender Committee is designated to support equal participation and recognition of women. Key tasks include consulting with women involved in farm-level cotton production, as well as other relevant community-level actors, raising awareness with Producer Management and farming communities of locally specific gender dynamics, and working with Producer Management to develop measures to respond to the identified challenges and opportunities.</t>
+          <t>Payment of the Premium is reported in the traceability platform and meets at least the required minimum for crops with a prescribed minimum.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>1.5.2</t>
+          <t>3.1.2</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>In close collaboration with the Gender Lead or Gender Committee, the Producer implements recommended measures to enhance gender equality and inclusion as part of the activity and monitoring plans.</t>
+          <t>Responsible Certificate Holders have contracts or signed agreements specifying the amounts to be paid and the terms and conditions of the payment by period/cycle. Premium is not paid in kind and is paid in full according to the payment terms per crop specified in the Premium Annex.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>1.6.1</t>
+          <t>3.1.3</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>The Producer demonstrates collaboration or engagement with other relevant stakeholders on locally relevant sustainability issues.</t>
+          <t>Group management distributes at least 40% of the premium in cash or other monetary payments to group members in a timely and convenient manner prior to the next crop season, or at minimum annually in case of continuous harvest. Group members receive Premium on a pro-rata basis based upon volumes delivered. Group management documents and reports premium received by volume and in total, amount paid to group members, and how Premium is utilized by group management as a percentage of the total.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>1.7.1</t>
+          <t>3.1.4</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>The Producer is aware of locally relevant climate change adaptation measures and implements these in line with the activity and monitoring plans.</t>
+          <t>Any paid premium is spent to benefit producer or workers. Management documents Premium received by volume and in total, and distribution of the Premium as a percentage on amount received by volume on how it benefits producer or workers.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>1.7.2</t>
+          <t>4.1.1</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>The Producer is aware of locally relevant climate change mitigation measures and implements these in line with the activity and monitoring plans.</t>
+          <t>Plant varieties for planting, grafting, and renovation are selected based on quality, productivity, resistance to pests and diseases, and suitability for the climate during the lifetime of the plants. Planting materials are free of pests and diseases.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2.1.1</t>
+          <t>4.1.2</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Locally relevant practices that maximise crop diversity are implemented.</t>
+          <t>For new plantings, producers follow a well-established cropping system that considers various factors, including requirements of the variety used, geographical, ecological, and agronomic conditions, diversification and intercropping crops with different rooting depths and soil uses to enhance soil quality and health, and planting density.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2.1.2</t>
+          <t>4.1.3</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Locally relevant farming practices that maximise soil cover are implemented.</t>
+          <t>Based on IPM strategy, producers implement measures to prevent pests and diseases and to break their biological cycles, to support soil health and to improve weed management. Such measures can include intercropping.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2.1.3</t>
+          <t>4.2.1</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Locally relevant farming practices that minimize soil disturbance are implemented.</t>
+          <t>Producers implement a pruning cycle for the formation, maintenance, and rejuvenation of crops according to their needs, agroecological conditions, and applicable pruning guidelines.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2.1.4</t>
+          <t>4.3.1</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Based on soil and plant needs, optimum application of fertilisers aims to maximise benefits and minimise negative impacts, considering and selecting the right source of nutrient, right rate, right timing, and right place of application.</t>
+          <t>The certified crop is not genetically modified (GMO).</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2.1.5</t>
+          <t>4.4.1</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Alternative methods beyond synthetic fertilisers are used to address nutritional needs of plants and soils, and steps are taken to minimise the use of synthetic fertiliser over time.</t>
+          <t>Management conducts a soil assessment for a representative sample of areas, including erosion-prone areas and slope, soil structure, soil depth and soil horizons, densification of compaction areas, soil moisture and water level in the soil, drainage conditions, and levels of macronutrients and organic matter. The soil assessment is updated at least once every three years, and for annual crops, levels of macronutrients and organic matter are assessed annually.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2.2.1</t>
+          <t>4.4.2</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Irrigation methods, technologies, and timing are planned and implemented to improve irrigation efficiency and maximise water productivity.</t>
+          <t>Based on the soil assessment, management identifies soil management measures and includes these in the management plan to build up soil organic matter, increase on-farm nutrient recycling, and optimize soil moisture.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2.2.2</t>
+          <t>4.4.3</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Practices are implemented to effectively manage changing rainfall amount, intensity and timing.</t>
+          <t>Producers prioritize using farm-made organic fertilizers. If additional nutrients are needed, they supplement with other organic or inorganic fertilizers. Animal manure is hot composted to reduce risk and stored at least 25 meters from water bodies.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2.3.1</t>
+          <t>4.4.4</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Measures are implemented to protect water bodies, ensuring understanding of their importance and implementing practices to protect their quality, availability, and related biodiversity from adverse farming impacts.</t>
+          <t>The soil in the production area is covered using methods like cover crops, crop residues, or mulch to prevent exposure.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2.3.2</t>
+          <t>4.4.5</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Natural habitats and biodiversity are conserved, and steps are taken to enhance them over time in line with local or regional priorities.</t>
+          <t>Fertilizers are applied to ensure nutrients are available to crops at the appropriate times and locations, minimizing environmental contamination.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2.3.3</t>
+          <t>4.4.6</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Degraded areas on croplands are identified, and steps are taken to restore them over time in line with local or regional priorities.</t>
+          <t>Producers monitor and optimize the use of organic and inorganic fertilizers.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2.4.1</t>
+          <t>4.5.1</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>The Producer ensures that no cotton is grown on land converted from natural ecosystems after 31 December 2020, in line with the Better Cotton Land Conversion Reference Documents.</t>
+          <t>Management documents and implements an IPM strategy, developed by a competent professional, including for processing facilities. The strategy includes prevention, monitoring, threshold levels, and intervention measures. It is based on climate conditions, pest monitoring results, implemented actions, and pesticide application records. The IPM strategy is updated annually.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2.4.2</t>
+          <t>4.5.2</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Prior to any land conversion, the Better Cotton Land Conversion Assessment shall be undertaken to ensure that natural ecosystems and High Conservation Values (HCVs) are conserved. Resulting measures are fully implemented as part of the activity and monitoring plans in Principle 1.</t>
+          <t>Based on the IPM Strategy, producers improve natural ecosystems near crop production areas to provide habitat for natural enemies. Examples include creating insectaries, planting trees and shrubs that attract birds, bats, and pollinators, converting low-lying areas into small ponds with vegetation, and enhancing riparian areas and vegetation.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>3.1.1</t>
+          <t>4.6.1</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>A written Integrated Pest Management (IPM) strategy is developed and implemented which covers Indicators 3.1.2 - 3.1.6, supports improved awareness and implementation of IPM practices over time, and informs the activity and monitoring plans under Principle 1.</t>
+          <t>No agrochemicals are used that are on the Rainforest Alliance List of Prohibited Pesticides or List of Obsolete Pesticides, prohibited by applicable law, or not legally registered in the country where the farm is located. Producers use only agrochemicals sold by authorized vendors, in original and sealed packaging.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>3.1.2</t>
+          <t>4.6.2</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Methods are implemented that help grow a healthy crop, discourage the build-up of pest populations and diseases, and preserve and enhance populations of beneficial organisms.</t>
+          <t>Producers using pesticides on the Risk Mitigation list must implement all related practices described in the Farming Annex. Producers using pesticides under the Exceptional Use Policy must follow all respective practices detailed in this policy and adhere to the procedure for requesting and reporting exceptions as outlined in the annex.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>3.1.3</t>
+          <t>4.6.3</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Farmers are informed of appropriate seed varieties, based on consideration of suitability for local growing conditions and reducing susceptibility to key pests and/or diseases.</t>
+          <t>Pesticide handlers are trained annually in preparation and application. They use Personal Protective Equipment (PPE).</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>3.1.4</t>
+          <t>4.6.3</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Regular monitoring is conducted on crop health and levels of pests and beneficial organisms. Field observation and decision-making tools are used to determine when and how to control pests.</t>
+          <t>Pesticide handlers are trained annually in preparation and application, use Personal Protective Equipment (PPE) as specified by the product label or Material Safety Data Sheet (MSDS), or basic protective clothing based on risk when no information is available. PPE must be in good condition, washed and stored safely after use, and not taken into workers' housing. Single-use items are disposed of after one use. PPE is provided for free, and farm/group management records, monitors, and enforces PPE usage.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>3.1.5</t>
+          <t>4.6.4</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Farmers are aware of non-chemical methods for managing key pests, and their use is prioritised as part of the IPM strategy.</t>
+          <t>Pesticide handlers must bathe, change, and wash clothes after application. Management should provide them with a private area, water, soap, and, if possible, bathing facilities.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>3.1.6</t>
+          <t>4.6.5</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Pesticides are only used if a certain threshold of pests is reached. If pesticides are used, low toxicity active ingredients are preferred and they are selected and applied in a way to mitigate resistance.</t>
+          <t>Pesticides are prepared and applied according to the label, MSDS or security tag, or as recommended by an official national organization or a competent technician, especially with regards to safe transport to area of application, respecting the correct dosage, using appropriate equipment and techniques, appropriate weather conditions, respecting restricted entry intervals (REI), including warning signs in local language and informing potentially affected persons or communities in advance. When there is no other information, minimum restricted entry interval is 48 hours for WHO class II products and 12 hours for other products. When two or more products with different restricted entry intervals are used at the same time, the longest interval applies. Volume and dosage calculation methods are reviewed and refined to reduce the surplus mix and pesticide overuse. Pre-harvest intervals of pesticides as stipulated in the product’s MSDS, label or security tag or regulation by official organization are complied with. When two or more products with different pre-harvest intervals are used at the same time, the longest interval applies.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>3.1.4</t>
+          <t>4.6.6</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>The farmer applies pesticides only when pests reach a level where their damage to the crop is greater than the monetary cost of treatment, based on guidance and advice from a competent technician or training.</t>
+          <t>Mechanisms are in place to prevent contamination by pesticides, through spray drift or other means, from treated areas to other areas including all aquatic and terrestrial ecosystems and infrastructure. These mechanisms include non-crop vegetative barriers, non-application zones, or other effective measures.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>3.1.7</t>
+          <t>4.6.7</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>An Integrated Pest Management strategy is implemented which discourages the build-up of pest populations and crop diseases, supports beneficial organisms, includes regular monitoring of crop health, pests, diseases, and beneficial organisms, prioritises non-chemical methods, ensures pesticides are used only when defined pest thresholds are reached, and prioritises low toxicity active ingredients while managing plant resistance if pesticides are used.</t>
+          <t>Aerial application is only allowed under the conditions as outlined in the Farming Annex.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>3.2.1</t>
+          <t>4.6.8</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>All pesticides used are correctly labelled in at least one national or regional language and registered nationally for use on cotton. Pesticide mixtures may be used only if the mixture itself is registered or on-site mixtures of individually registered pesticides are permitted under local regulations.</t>
+          <t>Pesticide applications are recorded. Records include product brand name and active ingredient(s), date and time of application.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>3.3.1</t>
+          <t>4.6.8</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Highly Hazardous Pesticides (HHPs) shall not be used if they are listed in the Better Cotton Prohibited Pesticides List.</t>
+          <t>Pesticide applications are recorded, including product brand name and active ingredient(s), date and time of application, location and area (size) of application, dosage and volume (organic or inorganic), crop, name(s) of applicator(s), and target pest. Group management facilitates record keeping for group members when needed.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>3.3.2</t>
+          <t>4.6.9</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>A plan is implemented to phase out pesticides defined as carcinogenic (category 1a or 1b), mutagenic (category 1a or 1b) or reprotoxic (category 1a or 1b) by the Globally Harmonized System of Classification and Labelling of Chemicals (GHS) by 2028 or earlier.</t>
+          <t>Empty pesticide containers and application equipment are washed three times, with the rinsing water used in the final batch of the mix for crop application. After applying pesticides, application equipment is washed three times, and any leftover mix is diluted with ten times the amount of clean water and applied evenly on the treated field to minimize environmental and health impacts. Empty pesticide containers are stored securely until they can be disposed of safely through a formal collection or recycling program or returned to the supplier. If the supplier does not accept empty containers, they are cut or perforated to prevent reuse. Prohibited, obsolete, and expired pesticides are returned to the supplier or local authority. If no collection system is available, these products are labeled and stored safely and separately from other products in a locked space.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>3.4.1</t>
+          <t>4.6.10</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>If pesticides included in the Better Cotton High Environmental Hazard List are used, measures are implemented to mitigate environmental risks.</t>
+          <t>Agrochemicals and application equipment are stored in accordance with label instructions to ensure minimal negative impact on the environment and human health. Agrochemicals must remain in their original containers or packaging. Facilities for storing agrochemicals and application equipment should be dry, clean, and well-ventilated, constructed from non-absorbent materials, securely locked and accessible only by trained handlers, inaccessible to children, and separated from crops, food products, and packaging materials.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>3.5.1</t>
+          <t>4.6.11</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>It is ensured that any person who prepares and applies pesticides is healthy, skilled and trained in the application of pesticides, 18 or older, and not pregnant or nursing.</t>
+          <t>Agrochemicals and application equipment are stored in accordance with the label instructions and in a way that minimizes negative impact on the environment and human health. Agrochemicals are stored in their original containers or packaging. Facilities for storing agrochemicals and application equipment are dry, clean, well-ventilated and with a sound roof and impermeable floor, safely locked and accessible only by trained handlers, separated from crops, food products or packaging material, with an emergency spill kit, with visible and understandable safety warning signs and pictograms, and with an emergency procedure, eye-washing area and an emergency shower. For small farms in groups only requirement 4.6.10 applies.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>3.5.2</t>
+          <t>4.6.12</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Appropriate Personal Protective Equipment (PPE) is correctly used while using and handling pesticides.</t>
+          <t>An up-to-date pesticide stock inventory is available and maintained, including date of purchase.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>3.5.3</t>
+          <t>4.6.12</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Minimum Personal Protective Equipment (PPE) is correctly used while using and handling pesticides.</t>
+          <t>An up-to-date pesticide stock inventory is available and maintained, including date of purchase, product brand name and active ingredient with indication of chemicals on the Risk Mitigation list, volume, and date of expiration. For groups, this is only applicable for centralized stock.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>3.5.3</t>
+          <t>4.6.13</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Minimum Personal Protective Equipment (PPE) is correctly used while using and handling pesticides, which includes protection of the face and airways, limbs, and abdomen and genital area from dermal absorption, ingestion, and inhalation.</t>
+          <t>The equipment used for mixing and applying agrochemicals is calibrated at least once a year, after every maintenance session, and before it is used with a different type of agrochemical.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>3.5.4</t>
+          <t>4.7.1</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Steps are taken to increase the use of appropriate Personal Protective Equipment (PPE) amongst individuals using and handling pesticides.</t>
+          <t>Products are handled to maintain quality and quantity during harvest and post-harvest stages, including harvesting at the right time, minimizing plant damage, preventing contamination, avoiding moisture damage, storing in a cool, dry, dark, and well-ventilated place, maintaining and cleaning tools, and using suitable packaging materials.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>3.5.5</t>
+          <t>4.7.2</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Dedicated areas are available on the farm for using and handling pesticides and for storing and handling application equipment, fully complying with relevant legislation for the storage of pesticides, and all rinsate and runoff are completely captured to pose no contamination risk.</t>
+          <t>Measures are taken to comply with the maximum residue levels (MRLs) established by the production country and known destination countries, including adherence to agrochemical label instructions, obtaining residue information, taking actions if MRLs are exceeded, and informing the buyer if MRLs are exceeded.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>3.5.6</t>
+          <t>5.1.1</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Disposal of agrochemical containers minimises risks to human health and the environment, and farmers participate in recycling or return to supplier programmes where they exist.</t>
+          <t>Management commits to assess and address child labor, forced labor, discrimination, and workplace violence and harassment by coordinating the committees/persons responsible for managing grievances and gender issues, raising awareness on these issues with management and group staff at least once a year, and informing workers/group members in writing that these issues are not tolerated, with information visibly displayed at central locations at all times.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>3.5.7</t>
+          <t>5.1.2</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Farmers are aware of and adopt appropriate and less hazardous pesticide application techniques.</t>
+          <t>The management representative/committee includes mitigation measures in the management plan, using measures identified in the basic Risk Assessment and implementing corresponding measures.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>3.5.8</t>
+          <t>5.1.3</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Pesticide application minimises negative impacts by ensuring label requirements are followed, appropriate application equipment is used and calibrated correctly, appropriate weather conditions are taken into account, contamination is minimised and appropriate measures are in place to prevent harm to people and the environment, and restricted entry intervals are enforced after applying pesticides.</t>
+          <t>The committee/management representative monitors risks and the implementation of risk mitigation measures, reports potential cases of child labor, forced labor, discrimination, and workplace violence and harassment to the management and to the grievance committee, and monitors remediation activities.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>4.1.1</t>
+          <t>5.1.4</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Locally relevant good practices for seed selection, planting date, planting rate, row spacing, and crop growth are implemented.</t>
+          <t>The committee/management representative sets out in the management plan how to remediate cases of child labor, forced labor, discrimination, workplace violence and harassment, with confirmed cases remediated and documented following the Rainforest Alliance Remediation Protocol, ensuring safety and confidentiality of the victims throughout the process.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>4.1.1</t>
+          <t>5.1.5</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Locally relevant good practices for seed selection, planting date, planting rate, row spacing, crop growth, and weed management are implemented to increase the probability of producing high-quality fibre.</t>
+          <t>In year 1 of certification, the management representative/committee conducts the assess-and-address Risk Assessment for the medium/high risk issue(s), includes the corresponding mitigation measures in the management plan, implements these measures, and repeats the assess-and-address Risk Assessment at least every three years.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>4.1.2</t>
+          <t>5.1.6</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Locally relevant good picking, storing, and transportation practices are implemented to avoid contamination.</t>
+          <t>Management representative/committee provides training/awareness raising on child labor, forced labor, discrimination, and workplace violence and harassment to all group members or workers.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>1.1.5</t>
+          <t>5.1.7</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>All Producers are expected to comply with relevant labour law and regulations, applying the stricter set of requirements where laws and regulations do not align with requirements in the P&amp;C v.3.1.</t>
+          <t>Management puts in place measures to ensure children of group staff, group members, and group member workers attend school.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>5.1.1</t>
+          <t>5.1.8</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>A system is in place to regularly monitor risks and incidents of labour rights violations, with clearly identified individuals responsible for the monitoring system and representation of farmers and workers in the operation of the monitoring system. Where risks are identified, prompt actions are taken to address these and prevent their escalation.</t>
+          <t>The management assures good functioning of the assess-and-address system by conducting a yearly assessment of the system for the relevant issue(s) based on effective implementation of mitigation measures, effective training on relevant topics, effective cooperation with external actors, effective monitoring of the system, and effective internal collaboration on topics.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>5.1.2</t>
+          <t>5.2.1</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>All workers have access to impartial, effective and secure channels to raise concerns about rights violations and have these addressed.</t>
+          <t>Workers can form and join unions or workers' organizations of their choice and participate in collective bargaining without employer approval, as per applicable law. Workers’ representatives are elected democratically in regular free and fair elections. Management has a written policy on workers' rights and ensures workers understand it, displaying it visibly in the workplace at all times. If laws restrict freedom of association and collective bargaining, management supports alternative methods for independent and free association, bargaining, and dialogue with workers.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>5.1.3</t>
+          <t>5.2.2</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Where labour rights violations occur, victims have access to protection and remediation.</t>
+          <t>Workers are protected from discrimination or retaliation due to union activities. Management cannot punish, bribe, or influence union members or representatives. Termination records include reasons and union affiliations. Management must not interfere in workers' organizations, their elections, or duties.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>5.1.3</t>
+          <t>5.2.3</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Where labour rights violations occur, victims have access to protection and remediation. Confidentiality and safety of victims are protected throughout the process.</t>
+          <t>Management provides workers’ representatives with reasonable paid time off to perform their representation functions and attend meetings. When necessary, management offers these representatives reasonable facilities, including meeting space, communication tools, and childcare. Management allows worker organizations and/or trade unions access to a notice board for posting information about their activities. Management establishes dialogue with freely chosen workers’ representatives to collectively discuss and address working conditions and terms of employment. Management maintains records of the minutes from meetings with worker organizations and/or trade unions.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>5.1.4</t>
+          <t>5.3.1</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Workers have access to an impartial, effective, and secure complaints hotline or other grievance mechanism. Any victims of labour rights violations shall be able to access support and remedy.</t>
+          <t>Workers employed for 3 consecutive months or more must have a written contract signed by both parties. Those employed for less than 3 months must have at least a verbal contract, with the employer keeping records of these contracts. Written contracts for workers employed 3 consecutive months or more include job duties, job location, and working hours.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>5.2.1</t>
+          <t>5.3.2</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Farmers and workers understand their fundamental principles and rights at work, including their rights to freedom of association and collective bargaining, a safe and healthy working environment, and protection from discrimination, forced or compulsory labour, and child labour.</t>
+          <t>There are no policies and/or arrangements to reduce workers' pay or benefits, such as using temporary workers for permanent tasks.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>5.3.1</t>
+          <t>5.3.3</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Children and young workers carry out only safe and age-appropriate tasks, in accordance with ILO Conventions 138 and 182.</t>
+          <t>Management and producers adhere to collective bargaining agreements relevant to the Rainforest Alliance Standard. Workers are paid at least the applicable minimum wage or the wage stipulated in a CBA, whichever is higher. For production quota or piece work, the payment must meet at least the minimum wage, based on a 48-hour working week or the national legal working hours limit, whichever is lower.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>5.4.1</t>
+          <t>5.3.4</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Workers understand and freely agree to the terms and conditions of work prior to starting (via verbal or written agreements) and any changes in conditions or nature of work (for example, overtime).</t>
+          <t>Deductions from wages for social security are only allowed if specified by applicable law or CBA. Voluntary deductions, like advance payments or loans, require worker consent. Employers must handle these remittances fully and in a timely manner. Disciplinary wage deductions are prohibited. Deductions for tools or gear are not allowed unless legally permitted. In-kind benefits must comply with the law and cannot exceed 30% of total pay.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>5.4.2</t>
+          <t>5.3.5</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Recruitment fees or related costs are not collected directly or indirectly from workers by an employer or other third party.</t>
+          <t>Workers receive payments at regular intervals as agreed upon by both the worker and the employer, with a minimum frequency of once per month. Detailed records are kept for each worker, including hours worked (both regular and overtime), production volume (where applicable), wage calculations, deductions, and payments made. Workers are provided with proof of payment (either physical or electronic) that includes this information.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>5.4.3</t>
+          <t>5.3.6</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Workers do not face threats or menace of penalty at any point during the whole work cycle, beginning from recruitment through to termination.</t>
+          <t>Work of equal value receives equal remuneration, free from discrimination on grounds such as gender, worker type, ethnicity, age, color, religion, political opinion, nationality, social origin, or other factors.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>5.4.4</t>
+          <t>5.3.7</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Workers are free to leave their job, in line with verbal or written agreements.</t>
+          <t>If labor providers are used, records are kept including the name, contact details, and official registration number (if available). The labor provider is not engaged in fraudulent or coercive recruiting practices, compliant with applicable worker-related requirements 5.3 and 5.5 of this standard, and all recruitment fees are paid by the farm, not by workers.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>5.4.4</t>
+          <t>5.3.8</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Workers are free to leave their job in line with verbal or written agreements.</t>
+          <t>In countries without yearly minimum wage adjustments or CBA regulations, workers' wages are annually adjusted for inflation based on the national rate.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>5.5.1</t>
+          <t>5.4.1</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Farmers and workers are informed about their right to form or join an organisation of their own choosing and to collectively negotiate without interference or threat. All terms agreed upon through an effective collective bargaining process are respected by both parties.</t>
+          <t>Management annually assesses total remuneration (wages, bonuses, and benefits) for all workers against the Living Wage benchmark recommended by the Rainforest Alliance and in accordance with the Global Living Wage Coalition (GLWC) or any other accepted benchmark.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>5.5.2</t>
+          <t>5.5.1</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>There is no interference, discrimination or retaliation against workers related to the establishment or participation in organisations or collective bargaining.</t>
+          <t>Workers do not exceed eight regular working hours per day or 48 hours per week. They receive a 30-minute break after six consecutive hours and one full rest day after six consecutive working days. Guards do not exceed 60 hours per week or the applicable regulation, whichever is stricter.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>5.6.1</t>
+          <t>5.5.2</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>There is no discrimination in labour practices.</t>
+          <t>Overtime work is voluntary and allowed if it is requested timely, paid according to national law or CBA, whichever is higher; if neither exists, paid at least 1.5 times the regular wage, does not increase health and safety risks; incident rates during overtime are monitored and reduced if necessary, workers have safe transport home, the total work week does not exceed 60 hours, except in special cases, workers get a 30-minute break after 6 hours of work and at least 10 consecutive hours of rest per 24-hour period, and a record of regular and overtime hours is kept.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>5.6.1</t>
+          <t>5.5.3</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>There is no discrimination in labour practices, including hiring, tasks, compensation, access to training, promotion, termination, or retirement.</t>
+          <t>Permanent workers are entitled to paid parental leave, rights and benefits in accordance with applicable law. In absence of such law, workers receive paid maternity leave of at least 12 weeks, of which at least six weeks are taken after birth. They can return to their job after maternity leave on the same terms and conditions and without discrimination, loss of seniority or deduction of wages. Workers who are pregnant, nursing or have recently given birth are offered flexible working schedules and work site arrangements. Breastfeeding women have two additional 30-minute breaks per day and an appropriate space for breastfeeding to nurture the child.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>5.7.1</t>
+          <t>5.5.4</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Workers are paid at least minimum wages as per the statutory national or regional minimum applicable to agriculture or the collectively agreed upon wage, and wages are paid in a fair and timely manner.</t>
+          <t>Children of workers who are below the applicable minimum working age and accompanying their parents to the workplace must be provided with a safe area appropriate for their age and be under continuous supervision by adults at all times.</t>
         </is>
       </c>
     </row>
@@ -1720,1039 +1720,607 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Workers receive equal pay for equal work.</t>
+          <t>Management, with the assistance of staff or external experts possessing the necessary technical expertise, conducts an analysis of occupational health and safety risks within the certification scope.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>5.7.2</t>
+          <t>5.6.2</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Workers are paid at least minimum wages, or where local prevailing wages are below the minimum wage, the Producer implements a system to record average wages and takes steps to improve wages over time.</t>
+          <t>First aid boxes are available for treating work-related injuries, with free emergency care and hospital transport. They are located centrally at production, processing, and maintenance sites. Emergency showers and eyewashes are also present where needed. Trained first aid employees are on duty during work hours, and workers are informed about where to go for assistance in emergencies.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>5.8.1</t>
+          <t>5.6.3</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Workers are given adequate time and privacy for personal sanitation near the worksite.</t>
+          <t>Group members and workers know emergency procedures. Warning signs and safety instructions are clearly displayed. Workers can leave imminent danger situations without permission or penalty.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>5.8.2</t>
+          <t>5.6.4</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Workers have regular rest breaks with access to potable water. Where there is a risk of dehydration, heat stroke and related illnesses, access to shade is provided and other measures are implemented to prevent and address these issues.</t>
+          <t>Workers have access to sufficient and safe drinking water at all times through one of the following means: a public drinking water system, or drinking water provided by the management that is tested at least once every three years, or more frequently if the risk analysis as part of requirement 5.6.1 identifies a risk. Management maintains drinking water sources, distribution systems, and containers to prevent contamination. Drinking water stored in jars or containers is protected against contamination with a lid and is replaced with fresh drinking water at least every 24 hours.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>5.8.3</t>
+          <t>5.6.5</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Safety and health risks are identified, and measures are implemented to minimise these risks, including training for farmers, workers and relevant supervisors. If accidents or injuries occur, medical attention is provided, and steps are taken to prevent recurrence.</t>
+          <t>For small farms without safe drinking water, management trains and instructs group members on treating water by boiling, filtering, or chlorinating, and preventing contamination.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>5.9.1</t>
+          <t>5.6.6</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Workers have the right to a workplace free of violence and harassment during the whole work cycle, beginning from recruitment through to termination.</t>
+          <t>Workers always have access to sufficient and safe drinking water.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>5.9.2</t>
+          <t>5.6.6</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Any disciplinary actions are proportionate to the conduct in question, and the system in place includes fair warning principles.</t>
+          <t>Workers always have access to sufficient and safe drinking water.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>5.10.1</t>
+          <t>5.6.7</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Permanent and seasonal workers are informed of their right to have a written contract. If requested by the worker or if contracts are required by law, appropriate written contracts are provided.</t>
+          <t>Adequate, clean, and operational toilets and handwashing stations are available at or near agricultural production, processing, maintenance sites, offices, and workers' housing. Facilities are separated by gender when there are 10 or more workers, with urinals separate from toilets used by females. Safety and privacy for vulnerable groups are ensured through features such as well-lit and lockable facilities. Workers have access to these facilities whenever necessary.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>5.10.2</t>
+          <t>5.6.8</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Farmers are responsible for communicating the requirements under Criteria 5.1 - 5.9 to third parties and ensuring they are met if workers are employed through a third party.</t>
+          <t>Workers in hazardous conditions (e.g., under challenging terrain, with machines or with hazardous materials) use Personal Protective Equipment (PPE) provided for free and receive training on how to use them.</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>6.1.1</t>
+          <t>5.6.9</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>The Producer identifies, monitors and confirms key livelihoods focus areas based on engagement with individuals involved in farm-level cotton production and other relevant community-level stakeholders.</t>
+          <t>Machinery and other equipment are stored safely when not in use. All tools used by the workers are functional. Machines have clear, comprehensible instructions for safe usage, and hazardous parts are guarded or enclosed. Workers using these machines receive proper training and hold any necessary licenses required by law.</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>6.1.2</t>
+          <t>5.6.10</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Based on Indicator 6.1.1, locally relevant measures are taken that deliver improvements against the defined key livelihoods focus areas over time.</t>
+          <t>Female workers who are pregnant, nursing, or have recently given birth are not assigned to activities that pose a risk to their health or the health of their unborn child or infant. In cases of job reassignment, there is no reduction in remuneration. Pregnancy tests are not requested.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>6.1.1</t>
+          <t>5.6.11</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Locally relevant measures are taken that deliver improvements against the defined key livelihoods focus areas over time.</t>
+          <t>Workshops, storage areas, and processing facilities are safe, clean, well-lit, and ventilated. A written accident and emergency procedure includes marked fire exits, evacuation maps, and at least one annual emergency drill. Management informs workers about this procedure. Firefighting and spill remediation equipment are available, and workers are trained to use them. Only authorized personnel have access to workshops, storage, or processing facilities.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>1.1.1</t>
+          <t>5.6.12</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>A clear and locally relevant activity plan is developed and implemented for the Producer Unit, which is kept up to date, includes all activities, timelines, and responsibilities, and is reviewed at least annually considering monitoring findings.</t>
+          <t>Workers in workshops, storage areas, and processing facilities have clean, safe eating spaces protected from the sun and rain. Field workers can also eat in areas shielded from the sun and rain.</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>1.1.2</t>
+          <t>5.6.13</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>A monitoring plan is developed and implemented that defines the data and methods used to identify risks of non-conformities, measure progress, and understand the effectiveness of Producer Unit activities. Data and information are recorded, and learnings are used to inform the activity plan in Indicator 1.1.1.</t>
+          <t>Workers who handle hazardous agrochemicals undergo a medical examination annually. If they are regularly exposed to organophosphates or carbamate pesticides, the examination includes cholinesterase testing. Workers can access the results of their medical examination.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>1.1.3</t>
+          <t>5.7.1</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>A representative and inclusive sample of individuals involved in farm-level cotton production is consulted on their priorities and needs at least once a year. Key findings from this consultation are documented and considered in activity planning across all Principles and in setting priorities for continuous improvement.</t>
+          <t>Workers and their families housed or lodged on-site are provided with safe, clean, and adequate living quarters considering local conditions.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>1.2.1</t>
+          <t>5.7.2</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>In line with the Better Cotton Farm Data Requirements Document, accurate and complete Producer-level data is collected, validated, and reported.</t>
+          <t>Children living on-site and of school-going age attend school, either within safe walking distance or within reasonable traveling distance with safe transport available.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>1.2.2</t>
+          <t>5.7.3</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>In line with the Better Cotton Farm Data Requirements Document, accurate and complete farm-level data is collected, validated, and recorded.</t>
+          <t>Workers and their families housed on-site have safe, clean, and decent living conditions that consider local standards.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>1.3.1</t>
+          <t>5.7.4</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Specific focus areas and respective three-year targets for continuous improvement are set, and annual activities to work towards those targets are fully included and implemented as part of the overall activity and monitoring planning and implementation in Indicators 1.1.1 and 1.1.2. Focus areas consider locally relevant sustainability priorities, priorities resulting from monitoring activities (Indicator 1.1.2), and priorities from inclusive field-level consultation as per Indicator 1.1.3.</t>
+          <t>On-site living conditions have improved through measures taken to reduce extreme climate impacts like flooding and ensuring natural ventilation for airflow in all weather.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>1.3.2</t>
+          <t>5.8.1</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Specific and locally relevant sustainability targets are identified for continuous improvement, with activities implemented to achieve those targets and progress monitored as part of the overall management system.</t>
+          <t>Management respects the legal and customary rights of indigenous peoples and local communities, and any activities affecting their land, resources, or interests must have their free, prior, and informed consent.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>1.4.1</t>
+          <t>5.8.2</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>An effective programme is implemented to strengthen capacities of individuals involved in farm-level cotton production, with training and related activities focusing on locally relevant practices and innovations, informed by inclusive field-level consultations and feedback from previous trainings, and using effective approaches and tools.</t>
+          <t>The producer has legal or legitimate right to use the land, substantiated by ownership, leasehold, or other legal documents or by documentation of traditional or customary use rights.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>1.4.2</t>
+          <t>5.8.3</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Training and other related activities are designed to be inclusive and equally accessible to everyone who may benefit.</t>
+          <t>Management actively engages with communities located within or adjacent to the farm that may be impacted by its operations. Management identifies their concerns and interests related to these operations and informs them about the procedure for filing complaints in accordance with 1.5.1.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>1.4.3</t>
+          <t>6.1.1</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Participants understand the relevance and benefits of knowledge, skills, and practices promoted through training and other related activities.</t>
+          <t>From January 1st, 2014, onward, natural forests and other natural ecosystems have not been converted into agricultural production or other land uses.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>1.4.4</t>
+          <t>6.1.2</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>An effective programme is implemented to strengthen capacities of workers, with training and related activities focusing on locally relevant practices and innovations, informed by inclusive field-level consultations and feedback from previous trainings, using effective approaches and tools, and designed to be inclusive and equally accessible to all workers who may benefit.</t>
+          <t>Production or processing does not occur in protected areas or their officially designated buffer zones, except where it complies with applicable law.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>1.5.1</t>
+          <t>6.1.3</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>An individual Gender Lead or Gender Committee is designated to support equal participation and recognition of women, with key tasks including consulting with women and other relevant community-level actors to identify local gender equality challenges and opportunities, raising awareness of locally-specific gender dynamics, and working with Producer Management to develop measures to respond to identified challenges and opportunities.</t>
+          <t>The management plan includes mitigation measures from the Risk Assessment Tool for High Conservation Values. Management implements these measures.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>1.5.2</t>
+          <t>6.2.1</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>In close collaboration with the Gender Lead or Gender Committee, the Producer implements recommended measures to enhance gender equality and inclusion as part of the activity and monitoring plans.</t>
+          <t>Management develops and implements a plan to conserve natural ecosystems based on the map required in 1.2.9 and the natural ecosystems section of the Risk Assessment Tool in 1.3.1, and updates it annually.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>1.6.1</t>
+          <t>6.2.2</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>The Producer demonstrates collaboration or engagement with other relevant stakeholders on locally relevant sustainability issues.</t>
+          <t>Farms preserve all remnant forest trees unless they present hazards to people or infrastructure, and manage other native trees sustainably to ensure the same quantity and quality of trees is maintained.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>1.7.1</t>
+          <t>6.2.3</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>The Producer is aware of locally relevant climate change adaptation measures and implements these in line with the activity and monitoring plans.</t>
+          <t>Producers maintain and management monitors natural vegetation cover and reports annually. If there is less than 10% of the total area under natural vegetation cover or less than 15% for farms growing shade-tolerant crops, management sets targets and takes actions for farms to reach these thresholds as required in 6.2.4.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>1.7.2</t>
+          <t>6.2.4</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>The Producer is aware of locally relevant climate change mitigation measures and implements these in line with the activity and monitoring plans.</t>
+          <t>There is natural vegetation cover on at least 10% of the total area for farms growing non-shade tolerant crops and on at least 15% of the total area for farms growing shade-tolerant crops.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>3.5.1</t>
+          <t>6.3.1</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>It is ensured that any person who prepares and applies pesticides is healthy, skilled and trained in the application of pesticides, 18 or older, and not pregnant or nursing.</t>
+          <t>Farms maintain existing riparian buffers adjacent to aquatic ecosystems.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>3.5.2</t>
+          <t>6.3.2</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Appropriate Personal Protective Equipment (PPE) is correctly used when handling pesticides.</t>
+          <t>Producers maintain additional safeguards for the protection of drinking water if the farm is located closer than 50m from a river, lake, or other water body frequently used as the main source of drinking water, including maintaining or establishing a riparian buffer at least 10m wide, adding an outer 20m non-application zone, and an additional 20m zone where pesticides are only applied through mechanical, hand-assisted, or targeted application.</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>3.5.3</t>
+          <t>6.3.3</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Minimum Personal Protective Equipment (PPE) is correctly used while using and handling pesticides, which includes protection of the face and airways, limbs, and abdomen and genital area from dermal absorption, ingestion, and inhalation.</t>
+          <t>Aquatic ecosystems are surrounded by riparian buffers with specified width parameters.</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>3.5.4</t>
+          <t>6.4.1</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Steps are taken to increase the use of appropriate Personal Protective Equipment (PPE) amongst individuals using and handling pesticides.</t>
+          <t>Threatened animals and plants are not hunted, killed, fished, collected, or trafficked. Producers and workers do not hunt other animals, except under specified conditions.</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>5.1.1</t>
+          <t>6.4.2</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>A system is in place to regularly monitor risks and incidents of labour rights violations, with responsible individuals clearly identified and farmers and workers represented in the operation of the monitoring system. Where risks are identified, prompt actions are taken to address these and prevent their escalation.</t>
+          <t>Producers do not keep wildlife in captivity. Captive wild animals present on the farm before the initial certification date are sent to professional shelters or may be kept only for non-commercial purposes for the rest of their lives.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>5.1.2</t>
+          <t>6.4.3</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>All workers have access to impartial, effective and secure channels to raise concerns about rights violations and have these addressed.</t>
+          <t>Producers avoid intentionally introducing or releasing invasive species. Producers do not dispose of existing invasive species or their parts in aquatic ecosystems.</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>5.1.3</t>
+          <t>6.4.4</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Where labour rights violations occur, victims have access to protection and remediation. Confidentiality and safety of victims are protected throughout the process.</t>
+          <t>Producers do not use wildlife for processing or harvesting of any crop.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>5.1.3</t>
+          <t>6.4.5</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Where labour rights violations occur, victims have access to protection and remediation. Confidentiality and safety of victims are protected throughout the process.</t>
+          <t>Erosion by water and wind is reduced through practices such as re-vegetation of steep areas and terracing.</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>5.1.4</t>
+          <t>6.4.6</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Workers have access to an impartial, effective and secure complaints hotline or other grievance mechanism. Any victims of labour rights violations shall be able to access support and remedy.</t>
+          <t>Fire is not used for preparing or cleaning fields, except when specifically justified in the IPM plan.</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>5.2.1</t>
+          <t>6.5.1</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Farmers and workers understand their fundamental principles and rights at work, including their rights to freedom of association and collective bargaining, a safe and healthy working environment, and protection from discrimination, forced or compulsory labour and child labour.</t>
+          <t>Management complies with the applicable law for withdrawal of surface or groundwater for agricultural, domestic or processing purposes.</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>5.3.1</t>
+          <t>6.5.1</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Children and young workers carry out only safe and age-appropriate tasks in accordance with ILO Conventions 138 and 182 and as set out in Table 1.</t>
+          <t>Management complies with the applicable law for withdrawal of surface or groundwater for agricultural, domestic or processing purposes. If required, compliance is demonstrated through a license or permit (or a pending request).</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>5.4.3</t>
+          <t>6.5.2</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Workers do not face threats or menace of penalty at any point during the whole work cycle, beginning from recruitment through to termination, including withholding of wages or documents, restrictions of movement or threats of violence.</t>
+          <t>Irrigation and water distribution systems are maintained to maximize crop yields while reducing water wastage, soil erosion, and salinization.</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>5.6.1</t>
+          <t>6.5.3</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>There is no discrimination in labour practices, including, but not limited to, hiring, tasks, compensation, access to training, promotion, termination or retirement.</t>
+          <t>Irrigation and water distribution systems are managed to optimize crop productivity, considering factors such as crop evapotranspiration at different growth stages, soil conditions, and rainfall pattern. Producers record the amount of water used for irrigation starting from year one onwards.</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>5.7.1</t>
+          <t>6.5.4</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Workers are paid at least minimum wages as per the statutory national or regional minimum applicable to agriculture or the collectively agreed upon wage. Wages are paid in a fair and timely manner.</t>
+          <t>Management takes measures to reduce the use of processing water per unit of product. Water use and reduction are monitored and documented from year one onwards.</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>5.7.2</t>
+          <t>6.5.5</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Workers are paid at least minimum wages, or where local prevailing wages are below the minimum wage, the Producer implements a system to record average wages and takes steps to improve wages over time.</t>
+          <t>Producers use rainwater harvesting for irrigation and/or other agricultural purposes.</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>5.8.1</t>
+          <t>6.5.6</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Workers are given adequate time and privacy for personal sanitation near the worksite.</t>
+          <t>Producers participate in a local watershed committee or initiative and take action to help maintain or restore the watershed’s health as part of this collective process. The nature of the participation and actions taken are documented.</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>5.8.2</t>
+          <t>6.6.1</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Workers have regular rest breaks with access to potable water. Where there is a risk of dehydration, heat stroke and related illnesses, access to shade is provided and other measures are implemented to prevent and address these issues.</t>
+          <t>Tests for processing wastewater are conducted at all discharge points during the representative period(s) of operation, and results are documented. Wastewater from processing operations discharged into aquatic ecosystems meets legal wastewater quality parameters. In absence of these, it meets the wastewater parameters. Wastewater from processing operations may not be mixed with clean water to meet the parameters.</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>5.8.3</t>
+          <t>6.6.2</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Safety and health risks are identified, and measures are implemented to minimise these risks, including training for farmers, workers and relevant supervisors. If accidents or injuries occur, medical attention is provided, and steps are taken to prevent recurrence.</t>
+          <t>Human sewage, sludge, and sewage water are not used in production or processing. Treated sewage is only discharged into aquatic ecosystems. Treated discharge must meet legal wastewater quality standards or equivalent parameters if no legal standards exist.</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>5.9.1</t>
+          <t>6.6.3</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Workers have the right to a workplace free of violence and harassment during the whole work cycle, beginning from recruitment through to termination.</t>
+          <t>Wastewater from processing operations is only used on land after treatment to remove particulates and toxins. Treated wastewater for irrigation must meet specific parameters for both wastewater and irrigation.</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>6.1.1</t>
+          <t>6.7.1</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>The Producer identifies, monitors and confirms key livelihoods focus areas based on engagement with individuals.</t>
+          <t>Waste is managed to avoid health and safety risks. It is stored and disposed of only in designated areas, not in natural ecosystems. Non-organic waste is not left on land.</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>6.1.1</t>
+          <t>6.7.2</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>The Producer identifies, monitors and confirms key livelihoods focus areas based on engagement with individuals involved in farm-level cotton production and other relevant community-level stakeholders.</t>
+          <t>Producers do not burn waste, except in incinerators technically designed for the specific type of waste.</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>6.1.2</t>
+          <t>6.7.3</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Based on Indicator 6.1.1, locally relevant measures are taken that deliver improvements against the defined key livelihoods focus areas over time.</t>
+          <t>Producers segregate and recycle waste based on available waste management, recycling, and disposal options. Organic waste is composted, processed for use as organic or used as input for other processes. Not applicable to small farms in groups.</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>1.1.1</t>
+          <t>6.8.1</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>A clear and locally relevant activity plan is developed and implemented for the Producer Unit, which is kept up to date, includes all activities, timelines, and responsibilities, and is reviewed at least annually considering monitoring findings.</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>1.3.1</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>Specific focus areas and respective three-year targets for continuous improvement are set, and annual activities to work towards those targets are fully included and implemented as part of the overall activity and monitoring planning and implementation in Indicators 1.1.1 and 1.1.2. Focus areas consider locally relevant sustainability priorities, priorities resulting from monitoring activities, and priorities from inclusive field-level consultation and from the work conducted by the Gender Lead or Gender Committee.</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>1.3.2</t>
-        </is>
-      </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>Specific and locally relevant sustainability targets are identified to focus on for continuous improvement. Activities to achieve those targets are implemented and progress monitored.</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>1.3.2</t>
-        </is>
-      </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>Specific and locally relevant sustainability targets are identified for continuous improvement, with activities implemented and progress monitored as part of the overall management system.</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>1.4.1</t>
-        </is>
-      </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>An effective programme is implemented to strengthen capacities of individuals involved in farm-level cotton production, focusing on locally relevant practices and innovations, informed by inclusive field-level consultations and feedback from previous trainings, using effective approaches and tools to drive field-level impact.</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="inlineStr">
-        <is>
-          <t>1.6.1</t>
-        </is>
-      </c>
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>The Producer demonstrates collaboration or engagement with other relevant stakeholders on locally relevant sustainability issues.</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>1.7.1</t>
-        </is>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>The Producer is aware of locally relevant climate change adaptation measures and implements these in line with the activity and monitoring plans.</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t>1.7.2</t>
-        </is>
-      </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>The Producer is aware of locally relevant climate change mitigation measures and implements these in line with the activity and monitoring plans.</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t>2.1.1</t>
-        </is>
-      </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>Locally relevant practices that maximise crop diversity are implemented.</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>2.1.2</t>
-        </is>
-      </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>Locally relevant farming practices that maximise soil cover are implemented.</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>2.1.3</t>
-        </is>
-      </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>Locally relevant farming practices that minimise soil disturbance are implemented.</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>2.1.4</t>
-        </is>
-      </c>
-      <c r="B169" t="inlineStr">
-        <is>
-          <t>Based on soil and plant needs, optimum application of fertilisers aims to maximise benefits and minimise negative impacts, considering and selecting the right source of nutrient, right rate, right timing, and right place of application.</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>2.1.5</t>
-        </is>
-      </c>
-      <c r="B170" t="inlineStr">
-        <is>
-          <t>Alternative methods beyond synthetic fertilisers are used to address nutritional needs of plants and soils, with steps taken to minimise the use of synthetic fertiliser over time.</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>2.2.1</t>
-        </is>
-      </c>
-      <c r="B171" t="inlineStr">
-        <is>
-          <t>Irrigation methods, technologies and timing are planned and implemented to improve irrigation efficiency and maximise water productivity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>2.2.2</t>
-        </is>
-      </c>
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>Practices are implemented to effectively manage changing rainfall amount, intensity and timing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>2.2.2</t>
-        </is>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>Practices are implemented to effectively manage changing rainfall amount, intensity and timing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>2.3.1</t>
-        </is>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>Measures are implemented to protect water bodies.</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>2.3.2</t>
-        </is>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>Natural habitats and biodiversity are conserved, and steps are taken to enhance them over time in line with local or regional priorities.</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>2.3.3</t>
-        </is>
-      </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>Degraded areas on croplands are identified, and steps are taken to restore them over time in line with local or regional priorities.</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>2.4.1</t>
-        </is>
-      </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>The Producer ensures that no cotton is grown on land converted from natural ecosystems after 31 December 2020, in line with the Better Cotton Land Conversion Reference Documents.</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>2.4.2</t>
-        </is>
-      </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>Prior to any land conversion, the Better Cotton Land Conversion Assessment shall be undertaken to ensure that natural ecosystems and High Conservation Values (HCVs) are conserved. Resulting measures are fully implemented as part of the activity and monitoring plans in Principle 1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>3.1.1</t>
-        </is>
-      </c>
-      <c r="B179" t="inlineStr">
-        <is>
-          <t>A written Integrated Pest Management (IPM) strategy is developed and implemented which covers Indicators 3.1.2 - 3.1.6, supports improved awareness and implementation of IPM practices over time, and informs the activity and monitoring plans under Principle 1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>3.1.2</t>
-        </is>
-      </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>Methods are implemented that help grow a healthy crop, discourage the build-up of pest populations and diseases, and preserve and enhance populations of beneficial organisms.</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>3.1.3</t>
-        </is>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>Farmers are informed of appropriate seed varieties, based on consideration of suitability for local growing conditions and reducing susceptibility to key pests and/or diseases.</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>3.1.4</t>
-        </is>
-      </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>Regular monitoring is conducted on crop health and levels of pests and beneficial organisms. Field observation and decision-making tools are used to determine when and how to control pests.</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>3.1.5</t>
-        </is>
-      </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>Farmers are aware of non-chemical methods (for example, biological, physical and cultural) for managing key pests, and their use is prioritised as part of the IPM strategy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>3.1.6</t>
-        </is>
-      </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>Pesticides are only used if a certain threshold of pests is reached. If pesticides are used, low toxicity active ingredients are preferred.</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>3.1.6</t>
-        </is>
-      </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>Pesticides are only used if a certain threshold of pests is reached. If pesticides are used, low toxicity active ingredients are preferred and they are selected and applied in a way to mitigate resistance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>3.1.7</t>
-        </is>
-      </c>
-      <c r="B186" t="inlineStr">
-        <is>
-          <t>An Integrated Pest Management strategy is implemented which discourages the build-up of pest populations and crop diseases, supports beneficial organisms, includes regular monitoring of crop health, pests, diseases and beneficial organisms, prioritises non-chemical methods, ensures pesticides are used only when defined pest thresholds are reached, prioritises low toxicity active ingredients and manages plant resistance if pesticides are used.</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>3.3.1</t>
-        </is>
-      </c>
-      <c r="B187" t="inlineStr">
-        <is>
-          <t>Highly Hazardous Pesticides (HHPs) shall not be used if they are listed in the Better Cotton Prohibited Pesticides List.</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>3.3.2</t>
-        </is>
-      </c>
-      <c r="B188" t="inlineStr">
-        <is>
-          <t>A plan is implemented to phase out pesticides defined as carcinogenic (category 1a or 1b), mutagenic (category 1a or 1b) or reprotoxic (category 1a or 1b) by the Globally Harmonized System of Classification and Labelling of Chemicals (GHS) by 2028 or earlier.</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t>3.4.1</t>
-        </is>
-      </c>
-      <c r="B189" t="inlineStr">
-        <is>
-          <t>If pesticides included in the Better Cotton High Environmental Hazard List are used, measures are implemented to mitigate environmental risks.</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>4.1.1</t>
-        </is>
-      </c>
-      <c r="B190" t="inlineStr">
-        <is>
-          <t>Locally relevant good practices for seed selection (where possible), planting date, planting rate, row spacing, crop growth and weed management are implemented to increase the probability of producing high-quality fibre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="inlineStr">
-        <is>
-          <t>5.8.2</t>
-        </is>
-      </c>
-      <c r="B191" t="inlineStr">
-        <is>
-          <t>Workers have regular rest breaks with access to potable water. Where there is a risk of dehydration, heat stroke and related illnesses, access to shade is provided and other measures are implemented to prevent and address these issues.</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>5.8.3</t>
-        </is>
-      </c>
-      <c r="B192" t="inlineStr">
-        <is>
-          <t>Safety and health risks are identified, and measures are implemented to minimise these risks (including training for farmers, workers and relevant supervisors). If accidents or injuries occur, medical attention is provided, and steps are taken to prevent recurrence.</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t>6.1.1</t>
-        </is>
-      </c>
-      <c r="B193" t="inlineStr">
-        <is>
-          <t>The Producer identifies, monitors, and confirms key livelihoods focus areas based on engagement with individuals involved in farm-level cotton production and other relevant community-level stakeholders.</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t>6.1.2</t>
-        </is>
-      </c>
-      <c r="B194" t="inlineStr">
-        <is>
-          <t>Based on 6.1.1, locally relevant measures are taken that deliver improvements against the defined key livelihoods focus areas over time.</t>
+          <t>Management documents the types of energy sources and the energy used for production and processing of certified product. This applies to Group Management only if groups use energy for processing.</t>
         </is>
       </c>
     </row>

</xml_diff>